<commit_message>
docs: update README and release notes to reflect new default policy deployment state; remove deprecated groups and adjust policy descriptions for clarity
</commit_message>
<xml_diff>
--- a/reference/CA_Baseline_-_Mirage.xlsx
+++ b/reference/CA_Baseline_-_Mirage.xlsx
@@ -1828,7 +1828,7 @@
       </c>
       <c r="N8" s="24" t="inlineStr">
         <is>
-          <t>AC_TokenProtection_Pilot</t>
+          <t>CA_TokenProtection_Pilot</t>
         </is>
       </c>
       <c r="O8" s="24" t="inlineStr">
@@ -1908,22 +1908,22 @@
       </c>
       <c r="AD8" s="24" t="inlineStr">
         <is>
-          <t>AC_ServiceAccount_Interactive</t>
+          <t>CA_ServiceAccount_Interactive</t>
         </is>
       </c>
       <c r="AE8" s="24" t="inlineStr">
         <is>
-          <t>AC_ServiceAccount</t>
+          <t>CA_ServiceAccount</t>
         </is>
       </c>
       <c r="AF8" s="24" t="inlineStr">
         <is>
-          <t>AC_ServiceAccount</t>
+          <t>CA_ServiceAccount</t>
         </is>
       </c>
       <c r="AG8" s="24" t="inlineStr">
         <is>
-          <t>AC_ServiceAccount</t>
+          <t>CA_ServiceAccount</t>
         </is>
       </c>
       <c r="AH8" s="24" t="inlineStr">
@@ -1975,202 +1975,202 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="F9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="G9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External, AC_TravelException</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External, CA_TravelException</t>
         </is>
       </c>
       <c r="H9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="I9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External, AC_DeviceCodeApproved</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External, CA_DeviceCodeApproved</t>
         </is>
       </c>
       <c r="J9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="K9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="L9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="M9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External, AUTOPILOT_DevicePrep</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External, AUTOPILOT_DevicePrep</t>
         </is>
       </c>
       <c r="N9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="P9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External, AUTOPILOT_DevicePrep</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External, AUTOPILOT_DevicePrep</t>
         </is>
       </c>
       <c r="Q9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="R9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="S9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="T9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="U9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="V9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount</t>
         </is>
       </c>
       <c r="W9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount</t>
         </is>
       </c>
       <c r="X9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount</t>
         </is>
       </c>
       <c r="Y9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount</t>
         </is>
       </c>
       <c r="Z9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount</t>
         </is>
       </c>
       <c r="AA9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount</t>
         </is>
       </c>
       <c r="AB9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="AC9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount, All Guest/External</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount, All Guest/External</t>
         </is>
       </c>
       <c r="AD9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_ServiceAccount_NonInteractive</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_ServiceAccount_NonInteractive</t>
         </is>
       </c>
       <c r="AE9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AF9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AG9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AH9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AI9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AJ9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AK9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AL9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass, AC_MSP_PartnerUsers (per-tenant)</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass, CA_MSP_PartnerUsers (per-tenant)</t>
         </is>
       </c>
       <c r="AM9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AN9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, BG_BreakGlass</t>
+          <t>CA_ExcludedFromCA, BG_BreakGlass</t>
         </is>
       </c>
       <c r="AO9" s="24" t="inlineStr">
         <is>
-          <t>AC_ExcludedFromCA, AC_ExcludedAgents</t>
+          <t>CA_ExcludedFromCA, CA_ExcludedAgents</t>
         </is>
       </c>
     </row>

</xml_diff>